<commit_message>
Sběr 2026-08-17: 1 přijato
</commit_message>
<xml_diff>
--- a/data/kola/2026-08-17/vysledky.xlsx
+++ b/data/kola/2026-08-17/vysledky.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,11 +47,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -107,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,14 +116,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -546,7 +538,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>chybí</t>
+          <t>odevzdal</t>
         </is>
       </c>
     </row>
@@ -556,25 +548,25 @@
           <t>Pokus 2</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>odevzdal</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Odevzdáno</t>
         </is>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <f>COUNTIF(B5:B6,"odevzdal")&amp;" / 2"</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Jak přenést do modelu:</t>
         </is>
@@ -644,171 +636,216 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Zkopírujte oblast B4:L8 a v modelu ji vložte do listu „IMPORT HLASOVACÍCH LÍSTKŮ“ na adresu B4 (vložit jako hodnoty).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Časová značka</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Uživatelské jméno</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Jméno a příjmení</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>AKCIE - ZAŘAZENÍ NOVÉHO TÉMATU č. 1</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>AKCIE - ZAŘAZENÍ NOVÉHO TÉMATU č. 2</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>AKCIE - VYŘAZENÍ STÁVAJÍCÍHO TÉMATU č. 1</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>AKCIE - VYŘAZENÍ STÁVAJÍCÍHO TÉMATU č. 2</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>DLUHOPISY - ZAŘAZENÍ NOVÉHO TÉMATU č. 1</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>DLUHOPISY - ZAŘAZENÍ NOVÉHO TÉMATU č. 2</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>DLUHOPISY - VYŘAZENÍ STÁVAJÍCÍHO TÉMATU č. 1</t>
         </is>
       </c>
-      <c r="L3" s="11" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>DLUHOPISY - VYŘAZENÍ STÁVAJÍCÍHO TÉMATU č. 2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="12" t="n">
+        <v>46251.33550925926</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>peta.simcak@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Pokus 1</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>pokus</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>hellow</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>world</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>hola</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>pokus1</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>3434234</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>heloween</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="n">
         <v>46251.32511574074</v>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>peta.simcak@outlook.cz</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Pokus 2</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>hello</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr"/>
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>world</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="H5" s="13" t="inlineStr"/>
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>pokus</t>
         </is>
       </c>
-      <c r="J4" s="14" t="inlineStr">
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>pokus 2</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>nepokus</t>
         </is>
       </c>
-      <c r="L4" s="14" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="15" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="15" t="n"/>
-      <c r="J5" s="15" t="n"/>
-      <c r="K5" s="15" t="n"/>
-      <c r="L5" s="15" t="n"/>
+      <c r="L5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
-      <c r="H6" s="15" t="n"/>
-      <c r="I6" s="15" t="n"/>
-      <c r="J6" s="15" t="n"/>
-      <c r="K6" s="15" t="n"/>
-      <c r="L6" s="15" t="n"/>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="14" t="n"/>
+      <c r="L6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="15" t="n"/>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="15" t="n"/>
-      <c r="J7" s="15" t="n"/>
-      <c r="K7" s="15" t="n"/>
-      <c r="L7" s="15" t="n"/>
+      <c r="B7" s="14" t="n"/>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="14" t="n"/>
+      <c r="H7" s="14" t="n"/>
+      <c r="I7" s="14" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="14" t="n"/>
+      <c r="L7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="15" t="n"/>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="15" t="n"/>
-      <c r="K8" s="15" t="n"/>
-      <c r="L8" s="15" t="n"/>
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="14" t="n"/>
+      <c r="G8" s="14" t="n"/>
+      <c r="H8" s="14" t="n"/>
+      <c r="I8" s="14" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="14" t="n"/>
+      <c r="L8" s="14" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kolo 2026-08-17 · lístků v bloku 1 z 5 · hodnocení jsou zapsána bez mezer (++ nikoli + +), jak je čte matice.</t>
+          <t>Kolo 2026-08-17 · lístků v bloku 2 z 5 · hodnocení jsou zapsána bez mezer (++ nikoli + +), jak je čte matice.</t>
         </is>
       </c>
     </row>

</xml_diff>